<commit_message>
fix: erorr in score function
</commit_message>
<xml_diff>
--- a/data/input/score_lms/251/2025-06-04_251_email-nhom-mh-hk.xlsx
+++ b/data/input/score_lms/251/2025-06-04_251_email-nhom-mh-hk.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\source code\automatic_work\data\input\score_lms\251\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\source code\automation-work\data\input\score_lms\251\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF1A9CD-FC10-49BD-B998-2D7DBA8D5E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056389CE-6D84-49A5-8AE2-ED115810855A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -3335,27 +3335,27 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R339"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="49.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7265625" style="1" customWidth="1"/>
     <col min="8" max="8" width="11" style="3" customWidth="1"/>
-    <col min="9" max="10" width="14.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.85546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" style="4" customWidth="1"/>
-    <col min="13" max="13" width="21.28515625" style="1" customWidth="1"/>
+    <col min="9" max="10" width="14.54296875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" style="4" customWidth="1"/>
+    <col min="13" max="13" width="21.26953125" style="1" customWidth="1"/>
     <col min="14" max="14" width="35" style="1" customWidth="1"/>
-    <col min="15" max="16" width="9.28515625" style="5" customWidth="1"/>
+    <col min="15" max="16" width="9.26953125" style="5" customWidth="1"/>
     <col min="17" max="17" width="10" style="4" customWidth="1"/>
-    <col min="18" max="18" width="24.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.54296875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>32</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -3576,7 +3576,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>44</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>56</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>56</v>
       </c>
@@ -3844,7 +3844,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>72</v>
       </c>
@@ -3897,7 +3897,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>72</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>81</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>88</v>
       </c>
@@ -4062,7 +4062,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>81</v>
       </c>
@@ -4118,7 +4118,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>93</v>
       </c>
@@ -4174,7 +4174,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>44</v>
       </c>
@@ -4230,7 +4230,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -4286,7 +4286,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>44</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>115</v>
       </c>
@@ -4398,7 +4398,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>124</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>133</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>135</v>
       </c>
@@ -4557,7 +4557,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>139</v>
       </c>
@@ -4610,7 +4610,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>143</v>
       </c>
@@ -4663,7 +4663,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>147</v>
       </c>
@@ -4716,7 +4716,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>149</v>
       </c>
@@ -4757,7 +4757,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>149</v>
       </c>
@@ -4810,7 +4810,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>159</v>
       </c>
@@ -4866,7 +4866,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>163</v>
       </c>
@@ -4919,7 +4919,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>168</v>
       </c>
@@ -4972,7 +4972,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>171</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>171</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>185</v>
       </c>
@@ -5131,7 +5131,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
@@ -5184,7 +5184,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>44</v>
       </c>
@@ -5240,7 +5240,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>44</v>
       </c>
@@ -5293,7 +5293,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>206</v>
       </c>
@@ -5405,7 +5405,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>206</v>
       </c>
@@ -5461,7 +5461,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>215</v>
       </c>
@@ -5514,7 +5514,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>215</v>
       </c>
@@ -5570,7 +5570,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>220</v>
       </c>
@@ -5623,7 +5623,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>215</v>
       </c>
@@ -5679,7 +5679,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>220</v>
       </c>
@@ -5735,7 +5735,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>220</v>
       </c>
@@ -5791,7 +5791,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>232</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>242</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>249</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>258</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>249</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>249</v>
       </c>
@@ -6109,7 +6109,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>258</v>
       </c>
@@ -6162,7 +6162,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>276</v>
       </c>
@@ -6218,7 +6218,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>276</v>
       </c>
@@ -6274,7 +6274,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>286</v>
       </c>
@@ -6327,7 +6327,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>286</v>
       </c>
@@ -6380,7 +6380,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>300</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>300</v>
       </c>
@@ -6486,7 +6486,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>306</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>276</v>
       </c>
@@ -6598,7 +6598,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>276</v>
       </c>
@@ -6651,7 +6651,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>320</v>
       </c>
@@ -6704,7 +6704,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>320</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>326</v>
       </c>
@@ -6813,7 +6813,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>330</v>
       </c>
@@ -6866,7 +6866,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>330</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>326</v>
       </c>
@@ -6975,7 +6975,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>330</v>
       </c>
@@ -7028,7 +7028,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>300</v>
       </c>
@@ -7081,7 +7081,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>300</v>
       </c>
@@ -7134,7 +7134,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>347</v>
       </c>
@@ -7190,7 +7190,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>347</v>
       </c>
@@ -7243,7 +7243,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>300</v>
       </c>
@@ -7296,7 +7296,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>351</v>
       </c>
@@ -7352,7 +7352,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>320</v>
       </c>
@@ -7405,7 +7405,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>320</v>
       </c>
@@ -7461,7 +7461,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>300</v>
       </c>
@@ -7514,7 +7514,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>320</v>
       </c>
@@ -7567,7 +7567,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>368</v>
       </c>
@@ -7620,7 +7620,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>372</v>
       </c>
@@ -7673,7 +7673,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>372</v>
       </c>
@@ -7729,7 +7729,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>375</v>
       </c>
@@ -7782,7 +7782,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>375</v>
       </c>
@@ -7835,7 +7835,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>383</v>
       </c>
@@ -7891,7 +7891,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>383</v>
       </c>
@@ -7944,7 +7944,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>387</v>
       </c>
@@ -7997,7 +7997,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>387</v>
       </c>
@@ -8050,7 +8050,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>383</v>
       </c>
@@ -8103,7 +8103,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>389</v>
       </c>
@@ -8156,7 +8156,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>394</v>
       </c>
@@ -8209,7 +8209,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>394</v>
       </c>
@@ -8265,7 +8265,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>394</v>
       </c>
@@ -8318,7 +8318,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>394</v>
       </c>
@@ -8374,7 +8374,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>394</v>
       </c>
@@ -8427,7 +8427,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>394</v>
       </c>
@@ -8480,7 +8480,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>405</v>
       </c>
@@ -8533,7 +8533,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>372</v>
       </c>
@@ -8589,7 +8589,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>405</v>
       </c>
@@ -8642,7 +8642,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>405</v>
       </c>
@@ -8695,7 +8695,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>405</v>
       </c>
@@ -8748,7 +8748,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>405</v>
       </c>
@@ -8801,7 +8801,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>411</v>
       </c>
@@ -8857,7 +8857,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>411</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>411</v>
       </c>
@@ -8969,7 +8969,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>411</v>
       </c>
@@ -9025,7 +9025,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>232</v>
       </c>
@@ -9078,7 +9078,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>411</v>
       </c>
@@ -9134,7 +9134,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>417</v>
       </c>
@@ -9190,7 +9190,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>417</v>
       </c>
@@ -9246,7 +9246,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>424</v>
       </c>
@@ -9299,7 +9299,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>306</v>
       </c>
@@ -9352,7 +9352,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>427</v>
       </c>
@@ -9405,7 +9405,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>387</v>
       </c>
@@ -9458,7 +9458,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>387</v>
       </c>
@@ -9511,7 +9511,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>387</v>
       </c>
@@ -9567,7 +9567,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>437</v>
       </c>
@@ -9620,7 +9620,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>437</v>
       </c>
@@ -9673,7 +9673,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>437</v>
       </c>
@@ -9726,7 +9726,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>258</v>
       </c>
@@ -9779,7 +9779,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>249</v>
       </c>
@@ -9832,7 +9832,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>452</v>
       </c>
@@ -9885,7 +9885,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>455</v>
       </c>
@@ -9938,7 +9938,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>452</v>
       </c>
@@ -9991,7 +9991,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>286</v>
       </c>
@@ -10047,7 +10047,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>286</v>
       </c>
@@ -10100,7 +10100,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>286</v>
       </c>
@@ -10153,7 +10153,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>286</v>
       </c>
@@ -10209,7 +10209,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>461</v>
       </c>
@@ -10265,7 +10265,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>286</v>
       </c>
@@ -10318,7 +10318,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>463</v>
       </c>
@@ -10371,7 +10371,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>463</v>
       </c>
@@ -10424,7 +10424,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>463</v>
       </c>
@@ -10480,7 +10480,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>463</v>
       </c>
@@ -10533,7 +10533,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>463</v>
       </c>
@@ -10586,7 +10586,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>463</v>
       </c>
@@ -10639,7 +10639,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>372</v>
       </c>
@@ -10695,7 +10695,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>479</v>
       </c>
@@ -10751,7 +10751,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>306</v>
       </c>
@@ -10804,7 +10804,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>481</v>
       </c>
@@ -10857,7 +10857,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>306</v>
       </c>
@@ -10910,7 +10910,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>389</v>
       </c>
@@ -10966,7 +10966,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>486</v>
       </c>
@@ -11022,7 +11022,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>461</v>
       </c>
@@ -11078,7 +11078,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>486</v>
       </c>
@@ -11131,7 +11131,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>389</v>
       </c>
@@ -11184,7 +11184,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>489</v>
       </c>
@@ -11237,7 +11237,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>389</v>
       </c>
@@ -11293,7 +11293,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>389</v>
       </c>
@@ -11346,7 +11346,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>481</v>
       </c>
@@ -11399,7 +11399,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>495</v>
       </c>
@@ -11452,7 +11452,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>481</v>
       </c>
@@ -11505,7 +11505,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>411</v>
       </c>
@@ -11561,7 +11561,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>495</v>
       </c>
@@ -11614,7 +11614,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>481</v>
       </c>
@@ -11667,7 +11667,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>405</v>
       </c>
@@ -11720,7 +11720,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>424</v>
       </c>
@@ -11776,7 +11776,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>424</v>
       </c>
@@ -11829,7 +11829,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>286</v>
       </c>
@@ -11882,7 +11882,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>276</v>
       </c>
@@ -11938,7 +11938,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>276</v>
       </c>
@@ -11991,7 +11991,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>276</v>
       </c>
@@ -12047,7 +12047,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>286</v>
       </c>
@@ -12100,7 +12100,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>452</v>
       </c>
@@ -12153,7 +12153,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>452</v>
       </c>
@@ -12206,7 +12206,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>452</v>
       </c>
@@ -12259,7 +12259,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>452</v>
       </c>
@@ -12315,7 +12315,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>452</v>
       </c>
@@ -12368,7 +12368,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>452</v>
       </c>
@@ -12421,7 +12421,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>509</v>
       </c>
@@ -12477,7 +12477,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>509</v>
       </c>
@@ -12533,7 +12533,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>515</v>
       </c>
@@ -12589,7 +12589,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>519</v>
       </c>
@@ -12636,7 +12636,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>528</v>
       </c>
@@ -12689,7 +12689,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>528</v>
       </c>
@@ -12745,7 +12745,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>528</v>
       </c>
@@ -12798,7 +12798,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>530</v>
       </c>
@@ -12854,7 +12854,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>424</v>
       </c>
@@ -12907,7 +12907,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>347</v>
       </c>
@@ -12960,7 +12960,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>424</v>
       </c>
@@ -13013,7 +13013,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>347</v>
       </c>
@@ -13069,7 +13069,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>424</v>
       </c>
@@ -13122,7 +13122,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>347</v>
       </c>
@@ -13175,7 +13175,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>375</v>
       </c>
@@ -13228,7 +13228,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>530</v>
       </c>
@@ -13281,7 +13281,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="185" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>548</v>
       </c>
@@ -13337,7 +13337,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="186" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>554</v>
       </c>
@@ -13390,7 +13390,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="187" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>463</v>
       </c>
@@ -13443,7 +13443,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="188" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>463</v>
       </c>
@@ -13496,7 +13496,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="189" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>463</v>
       </c>
@@ -13549,7 +13549,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>375</v>
       </c>
@@ -13602,7 +13602,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="191" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>558</v>
       </c>
@@ -13655,7 +13655,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="192" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>565</v>
       </c>
@@ -13708,7 +13708,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="193" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>572</v>
       </c>
@@ -13764,7 +13764,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="194" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>579</v>
       </c>
@@ -13817,7 +13817,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="195" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>585</v>
       </c>
@@ -13870,7 +13870,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="196" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>591</v>
       </c>
@@ -13923,7 +13923,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="197" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>596</v>
       </c>
@@ -13976,7 +13976,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="198" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>600</v>
       </c>
@@ -14032,7 +14032,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="199" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>605</v>
       </c>
@@ -14088,7 +14088,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>149</v>
       </c>
@@ -14129,7 +14129,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="201" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>612</v>
       </c>
@@ -14182,7 +14182,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="202" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>615</v>
       </c>
@@ -14238,7 +14238,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>622</v>
       </c>
@@ -14294,7 +14294,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>624</v>
       </c>
@@ -14347,7 +14347,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="205" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>630</v>
       </c>
@@ -14403,7 +14403,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="206" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>258</v>
       </c>
@@ -14459,7 +14459,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="207" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>383</v>
       </c>
@@ -14512,7 +14512,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="208" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>394</v>
       </c>
@@ -14565,7 +14565,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="209" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>394</v>
       </c>
@@ -14618,7 +14618,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="210" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>394</v>
       </c>
@@ -14671,7 +14671,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="211" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>383</v>
       </c>
@@ -14727,7 +14727,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="212" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>638</v>
       </c>
@@ -14780,7 +14780,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="213" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>647</v>
       </c>
@@ -14833,7 +14833,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>649</v>
       </c>
@@ -14886,7 +14886,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>652</v>
       </c>
@@ -14942,7 +14942,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>18</v>
       </c>
@@ -14995,7 +14995,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="217" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>18</v>
       </c>
@@ -15051,7 +15051,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>658</v>
       </c>
@@ -15107,7 +15107,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="219" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>660</v>
       </c>
@@ -15163,7 +15163,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>662</v>
       </c>
@@ -15216,7 +15216,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="221" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>660</v>
       </c>
@@ -15272,7 +15272,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="222" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>660</v>
       </c>
@@ -15325,7 +15325,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>675</v>
       </c>
@@ -15381,7 +15381,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>680</v>
       </c>
@@ -15434,7 +15434,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="225" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>680</v>
       </c>
@@ -15487,7 +15487,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="226" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>93</v>
       </c>
@@ -15540,7 +15540,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="227" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>691</v>
       </c>
@@ -15596,7 +15596,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>88</v>
       </c>
@@ -15649,7 +15649,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>695</v>
       </c>
@@ -15702,7 +15702,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="230" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>72</v>
       </c>
@@ -15758,7 +15758,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="231" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>696</v>
       </c>
@@ -15811,7 +15811,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>699</v>
       </c>
@@ -15864,7 +15864,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="233" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>703</v>
       </c>
@@ -15920,7 +15920,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="234" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>706</v>
       </c>
@@ -15973,7 +15973,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="235" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>652</v>
       </c>
@@ -16029,7 +16029,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="236" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>675</v>
       </c>
@@ -16082,7 +16082,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>675</v>
       </c>
@@ -16135,7 +16135,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>714</v>
       </c>
@@ -16188,7 +16188,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>88</v>
       </c>
@@ -16244,7 +16244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>717</v>
       </c>
@@ -16297,7 +16297,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="241" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>721</v>
       </c>
@@ -16350,7 +16350,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>722</v>
       </c>
@@ -16406,7 +16406,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="243" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>723</v>
       </c>
@@ -16462,7 +16462,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="244" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>728</v>
       </c>
@@ -16518,7 +16518,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="245" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>722</v>
       </c>
@@ -16571,7 +16571,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="246" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>703</v>
       </c>
@@ -16624,7 +16624,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="247" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>662</v>
       </c>
@@ -16680,7 +16680,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="248" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>733</v>
       </c>
@@ -16736,7 +16736,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="249" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>737</v>
       </c>
@@ -16792,7 +16792,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="250" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>742</v>
       </c>
@@ -16848,7 +16848,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="251" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>747</v>
       </c>
@@ -16901,7 +16901,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="252" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>747</v>
       </c>
@@ -16954,7 +16954,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="253" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>751</v>
       </c>
@@ -17010,7 +17010,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="254" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>755</v>
       </c>
@@ -17063,7 +17063,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>717</v>
       </c>
@@ -17116,7 +17116,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="256" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>728</v>
       </c>
@@ -17169,7 +17169,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="257" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>258</v>
       </c>
@@ -17222,7 +17222,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>763</v>
       </c>
@@ -17275,7 +17275,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="259" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>767</v>
       </c>
@@ -17328,7 +17328,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="260" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>773</v>
       </c>
@@ -17381,7 +17381,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="261" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>777</v>
       </c>
@@ -17434,7 +17434,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="262" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>777</v>
       </c>
@@ -17490,7 +17490,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="263" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>781</v>
       </c>
@@ -17543,7 +17543,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="264" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>787</v>
       </c>
@@ -17596,7 +17596,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>791</v>
       </c>
@@ -17649,7 +17649,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="266" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>795</v>
       </c>
@@ -17702,7 +17702,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="267" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>799</v>
       </c>
@@ -17755,7 +17755,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>804</v>
       </c>
@@ -17808,7 +17808,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="269" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>807</v>
       </c>
@@ -17861,7 +17861,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="270" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>809</v>
       </c>
@@ -17914,7 +17914,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="271" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>811</v>
       </c>
@@ -17970,7 +17970,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="272" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>816</v>
       </c>
@@ -18026,7 +18026,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="273" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>486</v>
       </c>
@@ -18079,7 +18079,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="274" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>389</v>
       </c>
@@ -18132,7 +18132,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="275" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>528</v>
       </c>
@@ -18188,7 +18188,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="276" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>389</v>
       </c>
@@ -18244,7 +18244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>330</v>
       </c>
@@ -18297,7 +18297,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>330</v>
       </c>
@@ -18350,7 +18350,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>823</v>
       </c>
@@ -18403,7 +18403,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>827</v>
       </c>
@@ -18459,7 +18459,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>829</v>
       </c>
@@ -18515,7 +18515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>832</v>
       </c>
@@ -18568,7 +18568,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="283" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>838</v>
       </c>
@@ -18624,7 +18624,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>843</v>
       </c>
@@ -18680,7 +18680,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="285" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>843</v>
       </c>
@@ -18733,7 +18733,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>838</v>
       </c>
@@ -18786,7 +18786,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="287" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>777</v>
       </c>
@@ -18842,7 +18842,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>850</v>
       </c>
@@ -18898,7 +18898,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="289" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>856</v>
       </c>
@@ -18951,7 +18951,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="290" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>860</v>
       </c>
@@ -19004,7 +19004,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="291" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>860</v>
       </c>
@@ -19057,7 +19057,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="292" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>864</v>
       </c>
@@ -19110,7 +19110,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="293" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>867</v>
       </c>
@@ -19166,7 +19166,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>872</v>
       </c>
@@ -19219,7 +19219,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="295" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>876</v>
       </c>
@@ -19272,7 +19272,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="296" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>880</v>
       </c>
@@ -19325,7 +19325,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="297" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>884</v>
       </c>
@@ -19378,7 +19378,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="298" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>886</v>
       </c>
@@ -19431,7 +19431,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="299" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>890</v>
       </c>
@@ -19484,7 +19484,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="300" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>894</v>
       </c>
@@ -19537,7 +19537,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="301" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>895</v>
       </c>
@@ -19590,7 +19590,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="302" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>897</v>
       </c>
@@ -19643,7 +19643,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="303" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>901</v>
       </c>
@@ -19696,7 +19696,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="304" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>829</v>
       </c>
@@ -19752,7 +19752,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="305" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>902</v>
       </c>
@@ -19805,7 +19805,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="306" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>763</v>
       </c>
@@ -19861,7 +19861,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="307" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>906</v>
       </c>
@@ -19914,7 +19914,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="308" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>910</v>
       </c>
@@ -19967,7 +19967,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="309" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>912</v>
       </c>
@@ -20023,7 +20023,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="310" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>912</v>
       </c>
@@ -20076,7 +20076,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="311" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>917</v>
       </c>
@@ -20129,7 +20129,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="312" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>777</v>
       </c>
@@ -20185,7 +20185,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="313" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>777</v>
       </c>
@@ -20238,7 +20238,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="314" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>777</v>
       </c>
@@ -20294,7 +20294,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="315" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>923</v>
       </c>
@@ -20350,7 +20350,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="316" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>923</v>
       </c>
@@ -20403,7 +20403,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="317" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>923</v>
       </c>
@@ -20459,7 +20459,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="318" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>923</v>
       </c>
@@ -20515,7 +20515,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="319" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>923</v>
       </c>
@@ -20568,7 +20568,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="320" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>923</v>
       </c>
@@ -20621,7 +20621,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="321" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>939</v>
       </c>
@@ -20674,7 +20674,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="322" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>941</v>
       </c>
@@ -20730,7 +20730,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="323" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>486</v>
       </c>
@@ -20783,7 +20783,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="324" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>486</v>
       </c>
@@ -20839,7 +20839,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="325" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>528</v>
       </c>
@@ -20895,7 +20895,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="326" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>528</v>
       </c>
@@ -20948,7 +20948,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="327" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>424</v>
       </c>
@@ -21001,7 +21001,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="328" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>320</v>
       </c>
@@ -21054,7 +21054,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="329" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>486</v>
       </c>
@@ -21107,7 +21107,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="330" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>300</v>
       </c>
@@ -21160,7 +21160,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="331" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>300</v>
       </c>
@@ -21216,7 +21216,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="332" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>171</v>
       </c>
@@ -21269,7 +21269,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="333" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>959</v>
       </c>
@@ -21322,7 +21322,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="334" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>171</v>
       </c>
@@ -21378,7 +21378,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="335" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>966</v>
       </c>
@@ -21434,7 +21434,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="336" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>968</v>
       </c>
@@ -21487,7 +21487,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="337" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>972</v>
       </c>
@@ -21540,7 +21540,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="338" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>171</v>
       </c>
@@ -21596,7 +21596,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="339" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>691</v>
       </c>
@@ -21650,6 +21650,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R339" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>